<commit_message>
Update Excel file and remove temporary file
Updated the contents of ccta-repo_*.xlsx and deleted the associated temporary file ~$ccta-repo_*.xlsx.
</commit_message>
<xml_diff>
--- a/ccta-repo_イメージ.xlsx
+++ b/ccta-repo_イメージ.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hirokishiga/Documents/development/ccta-repo-input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7280BE74-0A1E-CC4A-B86F-3A60A9C0E601}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E85F0A4F-AB2C-D249-ADD9-70BB3C8F11D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="540" yWindow="760" windowWidth="28300" windowHeight="16820" activeTab="1" xr2:uid="{7B77F844-70BA-3846-86BD-D352ACFF9C77}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="109">
   <si>
     <t>症例識別コード</t>
     <phoneticPr fontId="1"/>
@@ -977,6 +977,153 @@
     </rPh>
     <rPh sb="20" eb="21">
       <t xml:space="preserve">ミトメマセン </t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>高度石灰化により内腔評価困難です。</t>
+    <rPh sb="0" eb="5">
+      <t xml:space="preserve">コウドセッカイカ </t>
+    </rPh>
+    <rPh sb="8" eb="12">
+      <t xml:space="preserve">ナイクウヒョウカ </t>
+    </rPh>
+    <rPh sb="12" eb="14">
+      <t xml:space="preserve">コンナンデス </t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>motion artifactにより内腔評価困難です。</t>
+    <rPh sb="18" eb="22">
+      <t xml:space="preserve">ナイクウヒョウカ </t>
+    </rPh>
+    <rPh sb="22" eb="24">
+      <t xml:space="preserve">コンナンデス </t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>その他（プルダウン）</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>PFO SF(-)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>PFO SF(+)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>LA憩室</t>
+    <rPh sb="2" eb="4">
+      <t xml:space="preserve">ケイシツ </t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>その他（実際の記載）</t>
+    <rPh sb="4" eb="6">
+      <t xml:space="preserve">ジッサイン </t>
+    </rPh>
+    <rPh sb="7" eb="9">
+      <t xml:space="preserve">キサイ </t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>心房間にスリット様の造影所見を認めます。PFOを疑います。</t>
+    <rPh sb="0" eb="3">
+      <t xml:space="preserve">シンボウカン </t>
+    </rPh>
+    <rPh sb="8" eb="9">
+      <t xml:space="preserve">ヨウ </t>
+    </rPh>
+    <rPh sb="10" eb="14">
+      <t xml:space="preserve">ゾウエイショケン </t>
+    </rPh>
+    <rPh sb="15" eb="16">
+      <t xml:space="preserve">ミトメマス </t>
+    </rPh>
+    <rPh sb="24" eb="25">
+      <t xml:space="preserve">ウタガイマス </t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>心房間にスリット様の造影所見および造影剤の交通を認めます。PFOを疑います。</t>
+    <rPh sb="0" eb="3">
+      <t xml:space="preserve">シンボウカン </t>
+    </rPh>
+    <rPh sb="8" eb="9">
+      <t xml:space="preserve">ヨウ </t>
+    </rPh>
+    <rPh sb="10" eb="14">
+      <t xml:space="preserve">ゾウエイショケン </t>
+    </rPh>
+    <rPh sb="17" eb="20">
+      <t xml:space="preserve">ゾウエイザイノ </t>
+    </rPh>
+    <rPh sb="21" eb="23">
+      <t xml:space="preserve">コウツウ </t>
+    </rPh>
+    <rPh sb="24" eb="25">
+      <t xml:space="preserve">ミトメマス </t>
+    </rPh>
+    <rPh sb="33" eb="34">
+      <t xml:space="preserve">ウタガイマス </t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>LA前壁に憩室様の造影所見を認めます。</t>
+    <rPh sb="3" eb="4">
+      <t xml:space="preserve">ヘキ </t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t xml:space="preserve">ケイシツヨウノ </t>
+    </rPh>
+    <rPh sb="7" eb="8">
+      <t xml:space="preserve">ヨウ </t>
+    </rPh>
+    <rPh sb="9" eb="13">
+      <t xml:space="preserve">ゾウエイショケン </t>
+    </rPh>
+    <rPh sb="14" eb="15">
+      <t xml:space="preserve">ミトメマス </t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>冠動脈相にて左心耳内に造影欠損を認めます。</t>
+    <rPh sb="0" eb="3">
+      <t xml:space="preserve">カンドウミャクソウ </t>
+    </rPh>
+    <rPh sb="3" eb="4">
+      <t xml:space="preserve">ソウ </t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t xml:space="preserve">サシンジナイニ </t>
+    </rPh>
+    <rPh sb="8" eb="9">
+      <t xml:space="preserve">ミミ </t>
+    </rPh>
+    <rPh sb="9" eb="10">
+      <t xml:space="preserve">ナイニ </t>
+    </rPh>
+    <rPh sb="11" eb="15">
+      <t xml:space="preserve">ゾウエイケッソンヲ </t>
+    </rPh>
+    <rPh sb="16" eb="17">
+      <t xml:space="preserve">ミトメマス </t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>LAAT(+)</t>
+    <rPh sb="0" eb="2">
+      <t>LAAT</t>
     </rPh>
     <phoneticPr fontId="1"/>
   </si>
@@ -1780,16 +1927,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7DB68D2-6938-6E40-82A8-C31FB48B2CC1}">
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="20"/>
   <cols>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="5.7109375" customWidth="1"/>
+    <col min="3" max="3" width="7.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="39" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -1811,8 +1962,14 @@
       <c r="G1" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="2" spans="1:7">
+      <c r="H1" t="s">
+        <v>99</v>
+      </c>
+      <c r="I1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
         <v>49</v>
       </c>
@@ -1834,8 +1991,14 @@
       <c r="G2" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="3" spans="1:7">
+      <c r="H2" t="s">
+        <v>100</v>
+      </c>
+      <c r="I2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
       <c r="A3" t="s">
         <v>50</v>
       </c>
@@ -1857,8 +2020,14 @@
       <c r="G3" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="4" spans="1:7">
+      <c r="H3" t="s">
+        <v>101</v>
+      </c>
+      <c r="I3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
       <c r="A4" t="s">
         <v>51</v>
       </c>
@@ -1880,8 +2049,14 @@
       <c r="G4" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="5" spans="1:7">
+      <c r="H4" t="s">
+        <v>102</v>
+      </c>
+      <c r="I4" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
       <c r="B5" t="s">
         <v>37</v>
       </c>
@@ -1900,8 +2075,14 @@
       <c r="G5" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="6" spans="1:7">
+      <c r="H5" t="s">
+        <v>108</v>
+      </c>
+      <c r="I5" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
       <c r="B6" t="s">
         <v>38</v>
       </c>
@@ -1911,7 +2092,9 @@
       <c r="D6" t="s">
         <v>70</v>
       </c>
-      <c r="E6" s="16"/>
+      <c r="E6" s="16" t="s">
+        <v>97</v>
+      </c>
       <c r="F6" t="s">
         <v>62</v>
       </c>
@@ -1919,15 +2102,18 @@
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:9">
       <c r="B7" t="s">
         <v>39</v>
       </c>
       <c r="C7" s="15" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="8" spans="1:7">
+      <c r="E7" s="16" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
       <c r="B8" t="s">
         <v>40</v>
       </c>
@@ -1935,7 +2121,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:9">
       <c r="B9" t="s">
         <v>41</v>
       </c>
@@ -1943,7 +2129,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:9">
       <c r="B10" t="s">
         <v>42</v>
       </c>
@@ -1951,7 +2137,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:9">
       <c r="B11" t="s">
         <v>43</v>
       </c>
@@ -1959,13 +2145,13 @@
         <v>67</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:9">
       <c r="B12" t="s">
         <v>44</v>
       </c>
       <c r="C12" s="15"/>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:9">
       <c r="B13" t="s">
         <v>45</v>
       </c>
@@ -1976,7 +2162,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:9">
       <c r="B14" t="s">
         <v>46</v>
       </c>
@@ -1984,7 +2170,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:9">
       <c r="B15" t="s">
         <v>47</v>
       </c>
@@ -1995,7 +2181,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:9">
       <c r="B16" t="s">
         <v>48</v>
       </c>

</xml_diff>